<commit_message>
Add Screen size chager func and pass on global using for the package
</commit_message>
<xml_diff>
--- a/Plannif projet spaceshooter.xlsx
+++ b/Plannif projet spaceshooter.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Personel\SpaceShooter\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48A42FC9-307F-49E8-A252-01A43C70092C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Planning" sheetId="1" r:id="rId5"/>
+    <sheet name="Planning" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -268,29 +277,32 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/MM/yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FFFE0101"/>
       <name val="Roboto"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -301,79 +313,46 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF5B3F86"/>
-          <bgColor rgb="FF5B3F86"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <border>
         <left style="thin">
@@ -390,42 +369,66 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF5B3F86"/>
+          <bgColor rgb="FF5B3F86"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="Planning-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="Planning-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F51" displayName="Tâches_liées_à_un_événement" name="Tâches_liées_à_un_événement" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tâches_liées_à_un_événement" displayName="Tâches_liées_à_un_événement" ref="A1:F51">
   <tableColumns count="6">
-    <tableColumn name="Tâche" id="1"/>
-    <tableColumn name="État" id="2"/>
-    <tableColumn name="Propriétaire" id="3"/>
-    <tableColumn name="Étape" id="4"/>
-    <tableColumn name="Date limite" id="5"/>
-    <tableColumn name="Notes" id="6"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Tâche"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="État"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Propriétaire"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Étape"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Date limite"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Notes"/>
   </tableColumns>
-  <tableStyleInfo name="Planning-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Planning-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -615,24 +618,27 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F51"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="30.13"/>
-    <col customWidth="1" min="2" max="3" width="22.63"/>
-    <col customWidth="1" min="4" max="4" width="35.75"/>
-    <col customWidth="1" min="5" max="5" width="22.63"/>
-    <col customWidth="1" min="6" max="6" width="15.13"/>
+    <col min="1" max="1" width="30.140625" customWidth="1"/>
+    <col min="2" max="3" width="22.5703125" customWidth="1"/>
+    <col min="4" max="4" width="35.7109375" customWidth="1"/>
+    <col min="5" max="5" width="22.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1">
+    <row r="1" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -652,12 +658,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
+    <row r="2" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>8</v>
@@ -666,13 +672,13 @@
         <v>9</v>
       </c>
       <c r="E2" s="5">
-        <v>46266.0</v>
+        <v>46266</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
+    <row r="3" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -686,18 +692,18 @@
         <v>12</v>
       </c>
       <c r="E3" s="5">
-        <v>46259.0</v>
+        <v>46259</v>
       </c>
       <c r="F3" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
+    <row r="4" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>8</v>
@@ -706,18 +712,18 @@
         <v>6</v>
       </c>
       <c r="E4" s="5">
-        <v>46266.0</v>
+        <v>46266</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
+    <row r="5" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>8</v>
@@ -726,18 +732,18 @@
         <v>6</v>
       </c>
       <c r="E5" s="5">
-        <v>46266.0</v>
+        <v>46266</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1">
+    <row r="6" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>8</v>
@@ -746,18 +752,18 @@
         <v>6</v>
       </c>
       <c r="E6" s="5">
-        <v>46272.0</v>
+        <v>46272</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1">
+    <row r="7" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>8</v>
@@ -766,13 +772,13 @@
         <v>6</v>
       </c>
       <c r="E7" s="5">
-        <v>46272.0</v>
+        <v>46274</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
+    <row r="8" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -786,13 +792,13 @@
         <v>6</v>
       </c>
       <c r="E8" s="5">
-        <v>46272.0</v>
+        <v>46274</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
+    <row r="9" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -806,13 +812,13 @@
         <v>6</v>
       </c>
       <c r="E9" s="5">
-        <v>46272.0</v>
+        <v>46274</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1">
+    <row r="10" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>22</v>
       </c>
@@ -826,13 +832,13 @@
         <v>6</v>
       </c>
       <c r="E10" s="5">
-        <v>46272.0</v>
+        <v>46274</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" ht="22.5" customHeight="1">
+    <row r="11" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>23</v>
       </c>
@@ -846,18 +852,18 @@
         <v>6</v>
       </c>
       <c r="E11" s="5">
-        <v>46272.0</v>
+        <v>46274</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" ht="22.5" customHeight="1">
+    <row r="12" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>8</v>
@@ -866,18 +872,18 @@
         <v>25</v>
       </c>
       <c r="E12" s="5">
-        <v>46273.0</v>
+        <v>46273</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" ht="22.5" customHeight="1">
+    <row r="13" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>8</v>
@@ -886,18 +892,18 @@
         <v>24</v>
       </c>
       <c r="E13" s="5">
-        <v>46273.0</v>
+        <v>46273</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" ht="22.5" customHeight="1">
+    <row r="14" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>8</v>
@@ -906,13 +912,13 @@
         <v>24</v>
       </c>
       <c r="E14" s="5">
-        <v>46273.0</v>
+        <v>46273</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" ht="22.5" customHeight="1">
+    <row r="15" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -926,13 +932,13 @@
         <v>24</v>
       </c>
       <c r="E15" s="5">
-        <v>46274.0</v>
+        <v>46274</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" ht="22.5" customHeight="1">
+    <row r="16" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>31</v>
       </c>
@@ -946,13 +952,13 @@
         <v>32</v>
       </c>
       <c r="E16" s="5">
-        <v>46274.0</v>
+        <v>46274</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" ht="22.5" customHeight="1">
+    <row r="17" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>33</v>
       </c>
@@ -966,13 +972,13 @@
         <v>32</v>
       </c>
       <c r="E17" s="5">
-        <v>46274.0</v>
+        <v>46274</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" ht="22.5" customHeight="1">
+    <row r="18" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>35</v>
       </c>
@@ -986,13 +992,13 @@
         <v>32</v>
       </c>
       <c r="E18" s="5">
-        <v>46274.0</v>
+        <v>46274</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19" ht="22.5" customHeight="1">
+    <row r="19" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>37</v>
       </c>
@@ -1006,13 +1012,13 @@
         <v>32</v>
       </c>
       <c r="E19" s="5">
-        <v>46279.0</v>
+        <v>46279</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" ht="22.5" customHeight="1">
+    <row r="20" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>39</v>
       </c>
@@ -1026,13 +1032,13 @@
         <v>40</v>
       </c>
       <c r="E20" s="5">
-        <v>46279.0</v>
+        <v>46279</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="21" ht="22.5" customHeight="1">
+    <row r="21" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>41</v>
       </c>
@@ -1046,13 +1052,13 @@
         <v>40</v>
       </c>
       <c r="E21" s="5">
-        <v>46279.0</v>
+        <v>46279</v>
       </c>
       <c r="F21" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="22" ht="22.5" customHeight="1">
+    <row r="22" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>42</v>
       </c>
@@ -1066,13 +1072,13 @@
         <v>40</v>
       </c>
       <c r="E22" s="5">
-        <v>46281.0</v>
+        <v>46281</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="23" ht="22.5" customHeight="1">
+    <row r="23" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>43</v>
       </c>
@@ -1086,13 +1092,13 @@
         <v>40</v>
       </c>
       <c r="E23" s="5">
-        <v>46281.0</v>
+        <v>46281</v>
       </c>
       <c r="F23" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="24" ht="22.5" customHeight="1">
+    <row r="24" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>45</v>
       </c>
@@ -1106,13 +1112,13 @@
         <v>25</v>
       </c>
       <c r="E24" s="5">
-        <v>46286.0</v>
+        <v>46286</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="25" ht="22.5" customHeight="1">
+    <row r="25" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>47</v>
       </c>
@@ -1126,13 +1132,13 @@
         <v>25</v>
       </c>
       <c r="E25" s="5">
-        <v>46287.0</v>
+        <v>46287</v>
       </c>
       <c r="F25" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="26" ht="22.5" customHeight="1">
+    <row r="26" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>48</v>
       </c>
@@ -1146,13 +1152,13 @@
         <v>25</v>
       </c>
       <c r="E26" s="5">
-        <v>46286.0</v>
+        <v>46286</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="27" ht="22.5" customHeight="1">
+    <row r="27" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>49</v>
       </c>
@@ -1166,13 +1172,13 @@
         <v>25</v>
       </c>
       <c r="E27" s="5">
-        <v>46288.0</v>
+        <v>46288</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="28" ht="22.5" customHeight="1">
+    <row r="28" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>50</v>
       </c>
@@ -1186,13 +1192,13 @@
         <v>9</v>
       </c>
       <c r="E28" s="5">
-        <v>46286.0</v>
+        <v>46286</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="29" ht="22.5" customHeight="1">
+    <row r="29" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>52</v>
       </c>
@@ -1206,13 +1212,13 @@
         <v>53</v>
       </c>
       <c r="E29" s="5">
-        <v>46286.0</v>
+        <v>46286</v>
       </c>
       <c r="F29" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="30" ht="22.5" customHeight="1">
+    <row r="30" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>54</v>
       </c>
@@ -1226,13 +1232,13 @@
         <v>53</v>
       </c>
       <c r="E30" s="5">
-        <v>46286.0</v>
+        <v>46286</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="31" ht="22.5" customHeight="1">
+    <row r="31" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>56</v>
       </c>
@@ -1246,13 +1252,13 @@
         <v>54</v>
       </c>
       <c r="E31" s="5">
-        <v>46286.0</v>
+        <v>46286</v>
       </c>
       <c r="F31" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="32" ht="22.5" customHeight="1">
+    <row r="32" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>57</v>
       </c>
@@ -1266,13 +1272,13 @@
         <v>54</v>
       </c>
       <c r="E32" s="5">
-        <v>46287.0</v>
+        <v>46287</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="33" ht="22.5" customHeight="1">
+    <row r="33" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>58</v>
       </c>
@@ -1286,13 +1292,13 @@
         <v>9</v>
       </c>
       <c r="E33" s="5">
-        <v>46266.0</v>
+        <v>46266</v>
       </c>
       <c r="F33" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="34" ht="22.5" customHeight="1">
+    <row r="34" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>59</v>
       </c>
@@ -1306,13 +1312,13 @@
         <v>25</v>
       </c>
       <c r="E34" s="5">
-        <v>46293.0</v>
+        <v>46293</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="35" ht="22.5" customHeight="1">
+    <row r="35" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>61</v>
       </c>
@@ -1326,13 +1332,13 @@
         <v>25</v>
       </c>
       <c r="E35" s="5">
-        <v>46294.0</v>
+        <v>46294</v>
       </c>
       <c r="F35" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="36" ht="22.5" customHeight="1">
+    <row r="36" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>62</v>
       </c>
@@ -1346,13 +1352,13 @@
         <v>25</v>
       </c>
       <c r="E36" s="5">
-        <v>46294.0</v>
+        <v>46294</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="37" ht="22.5" customHeight="1">
+    <row r="37" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>64</v>
       </c>
@@ -1366,13 +1372,13 @@
         <v>65</v>
       </c>
       <c r="E37" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="F37" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="38" ht="22.5" customHeight="1">
+    <row r="38" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>66</v>
       </c>
@@ -1386,13 +1392,13 @@
         <v>65</v>
       </c>
       <c r="E38" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="39" ht="22.5" customHeight="1">
+    <row r="39" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>67</v>
       </c>
@@ -1406,13 +1412,13 @@
         <v>65</v>
       </c>
       <c r="E39" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="F39" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="40" ht="22.5" customHeight="1">
+    <row r="40" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>68</v>
       </c>
@@ -1426,13 +1432,13 @@
         <v>65</v>
       </c>
       <c r="E40" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="41" ht="22.5" customHeight="1">
+    <row r="41" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>69</v>
       </c>
@@ -1446,13 +1452,13 @@
         <v>65</v>
       </c>
       <c r="E41" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="F41" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="42" ht="22.5" customHeight="1">
+    <row r="42" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>70</v>
       </c>
@@ -1466,13 +1472,13 @@
         <v>65</v>
       </c>
       <c r="E42" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="43" ht="22.5" customHeight="1">
+    <row r="43" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>71</v>
       </c>
@@ -1486,13 +1492,13 @@
         <v>65</v>
       </c>
       <c r="E43" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="F43" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="44" ht="22.5" customHeight="1">
+    <row r="44" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>72</v>
       </c>
@@ -1506,13 +1512,13 @@
         <v>65</v>
       </c>
       <c r="E44" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="45" ht="22.5" customHeight="1">
+    <row r="45" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>73</v>
       </c>
@@ -1526,13 +1532,13 @@
         <v>65</v>
       </c>
       <c r="E45" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="F45" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="46" ht="22.5" customHeight="1">
+    <row r="46" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>74</v>
       </c>
@@ -1546,13 +1552,13 @@
         <v>65</v>
       </c>
       <c r="E46" s="5">
-        <v>46300.0</v>
+        <v>46300</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="47" ht="22.5" customHeight="1">
+    <row r="47" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>75</v>
       </c>
@@ -1566,13 +1572,13 @@
         <v>76</v>
       </c>
       <c r="E47" s="5">
-        <v>46301.0</v>
+        <v>46301</v>
       </c>
       <c r="F47" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="48" ht="22.5" customHeight="1">
+    <row r="48" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>78</v>
       </c>
@@ -1586,13 +1592,13 @@
         <v>76</v>
       </c>
       <c r="E48" s="5">
-        <v>46301.0</v>
+        <v>46301</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="49" ht="22.5" customHeight="1">
+    <row r="49" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>79</v>
       </c>
@@ -1606,13 +1612,13 @@
         <v>9</v>
       </c>
       <c r="E49" s="5">
-        <v>46308.0</v>
+        <v>46308</v>
       </c>
       <c r="F49" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="50" ht="22.5" customHeight="1">
+    <row r="50" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>80</v>
       </c>
@@ -1626,13 +1632,13 @@
         <v>9</v>
       </c>
       <c r="E50" s="5">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="51" ht="22.5" customHeight="1">
+    <row r="51" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>82</v>
       </c>
@@ -1646,130 +1652,130 @@
         <v>9</v>
       </c>
       <c r="E51" s="5">
-        <v>46309.0</v>
+        <v>46309</v>
       </c>
       <c r="F51" s="6" t="s">
         <v>83</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="E2:E51">
+  <dataValidations count="4">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="E2:E51" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>OR(NOT(ISERROR(DATEVALUE(E2))), AND(ISNUMBER(E2), LEFT(CELL("format", E2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B51">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B51" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Pas commencé,En cours,Bloqué,Terminé"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="A2:A51 F2:F51"/>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D51">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A2:A51 F2:F51" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" sqref="D2:D51" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Rien,Créer le projet MonoGame C#,Configurer Git et le dépôt GitHub,Créer les différents écrans,Créer le joueur,Créer les énemis,Créer systeme vague,Créer la base de donnée,Connecter le jeu à la base de données,Finir V1 du jeu,Après fase de testes"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A2"/>
-    <hyperlink r:id="rId2" ref="C2"/>
-    <hyperlink r:id="rId3" ref="A3"/>
-    <hyperlink r:id="rId4" ref="C3"/>
-    <hyperlink r:id="rId5" ref="A4"/>
-    <hyperlink r:id="rId6" ref="C4"/>
-    <hyperlink r:id="rId7" ref="A5"/>
-    <hyperlink r:id="rId8" ref="C5"/>
-    <hyperlink r:id="rId9" ref="A6"/>
-    <hyperlink r:id="rId10" ref="C6"/>
-    <hyperlink r:id="rId11" ref="A7"/>
-    <hyperlink r:id="rId12" ref="C7"/>
-    <hyperlink r:id="rId13" ref="A8"/>
-    <hyperlink r:id="rId14" ref="C8"/>
-    <hyperlink r:id="rId15" ref="A9"/>
-    <hyperlink r:id="rId16" ref="C9"/>
-    <hyperlink r:id="rId17" ref="A10"/>
-    <hyperlink r:id="rId18" ref="C10"/>
-    <hyperlink r:id="rId19" ref="A11"/>
-    <hyperlink r:id="rId20" ref="C11"/>
-    <hyperlink r:id="rId21" ref="A12"/>
-    <hyperlink r:id="rId22" ref="C12"/>
-    <hyperlink r:id="rId23" ref="A13"/>
-    <hyperlink r:id="rId24" ref="C13"/>
-    <hyperlink r:id="rId25" ref="A14"/>
-    <hyperlink r:id="rId26" ref="C14"/>
-    <hyperlink r:id="rId27" ref="A15"/>
-    <hyperlink r:id="rId28" ref="C15"/>
-    <hyperlink r:id="rId29" ref="A16"/>
-    <hyperlink r:id="rId30" ref="C16"/>
-    <hyperlink r:id="rId31" ref="A17"/>
-    <hyperlink r:id="rId32" ref="C17"/>
-    <hyperlink r:id="rId33" ref="A18"/>
-    <hyperlink r:id="rId34" ref="C18"/>
-    <hyperlink r:id="rId35" ref="A19"/>
-    <hyperlink r:id="rId36" ref="C19"/>
-    <hyperlink r:id="rId37" ref="A20"/>
-    <hyperlink r:id="rId38" ref="C20"/>
-    <hyperlink r:id="rId39" ref="A21"/>
-    <hyperlink r:id="rId40" ref="C21"/>
-    <hyperlink r:id="rId41" ref="A22"/>
-    <hyperlink r:id="rId42" ref="C22"/>
-    <hyperlink r:id="rId43" ref="A23"/>
-    <hyperlink r:id="rId44" ref="C23"/>
-    <hyperlink r:id="rId45" ref="A24"/>
-    <hyperlink r:id="rId46" ref="C24"/>
-    <hyperlink r:id="rId47" ref="A25"/>
-    <hyperlink r:id="rId48" ref="C25"/>
-    <hyperlink r:id="rId49" ref="A26"/>
-    <hyperlink r:id="rId50" ref="C26"/>
-    <hyperlink r:id="rId51" ref="A27"/>
-    <hyperlink r:id="rId52" ref="C27"/>
-    <hyperlink r:id="rId53" ref="A28"/>
-    <hyperlink r:id="rId54" ref="C28"/>
-    <hyperlink r:id="rId55" ref="A29"/>
-    <hyperlink r:id="rId56" ref="C29"/>
-    <hyperlink r:id="rId57" ref="A30"/>
-    <hyperlink r:id="rId58" ref="C30"/>
-    <hyperlink r:id="rId59" ref="A31"/>
-    <hyperlink r:id="rId60" ref="C31"/>
-    <hyperlink r:id="rId61" ref="A32"/>
-    <hyperlink r:id="rId62" ref="C32"/>
-    <hyperlink r:id="rId63" ref="A33"/>
-    <hyperlink r:id="rId64" ref="C33"/>
-    <hyperlink r:id="rId65" ref="A34"/>
-    <hyperlink r:id="rId66" ref="C34"/>
-    <hyperlink r:id="rId67" ref="A35"/>
-    <hyperlink r:id="rId68" ref="C35"/>
-    <hyperlink r:id="rId69" ref="A36"/>
-    <hyperlink r:id="rId70" ref="C36"/>
-    <hyperlink r:id="rId71" ref="A37"/>
-    <hyperlink r:id="rId72" ref="C37"/>
-    <hyperlink r:id="rId73" ref="A38"/>
-    <hyperlink r:id="rId74" ref="C38"/>
-    <hyperlink r:id="rId75" ref="A39"/>
-    <hyperlink r:id="rId76" ref="C39"/>
-    <hyperlink r:id="rId77" ref="A40"/>
-    <hyperlink r:id="rId78" ref="C40"/>
-    <hyperlink r:id="rId79" ref="A41"/>
-    <hyperlink r:id="rId80" ref="C41"/>
-    <hyperlink r:id="rId81" ref="A42"/>
-    <hyperlink r:id="rId82" ref="C42"/>
-    <hyperlink r:id="rId83" ref="A43"/>
-    <hyperlink r:id="rId84" ref="C43"/>
-    <hyperlink r:id="rId85" ref="A44"/>
-    <hyperlink r:id="rId86" ref="C44"/>
-    <hyperlink r:id="rId87" ref="A45"/>
-    <hyperlink r:id="rId88" ref="C45"/>
-    <hyperlink r:id="rId89" ref="A46"/>
-    <hyperlink r:id="rId90" ref="C46"/>
-    <hyperlink r:id="rId91" ref="A47"/>
-    <hyperlink r:id="rId92" ref="C47"/>
-    <hyperlink r:id="rId93" ref="A48"/>
-    <hyperlink r:id="rId94" ref="C48"/>
-    <hyperlink r:id="rId95" ref="A49"/>
-    <hyperlink r:id="rId96" ref="C49"/>
-    <hyperlink r:id="rId97" ref="A50"/>
-    <hyperlink r:id="rId98" ref="C50"/>
-    <hyperlink r:id="rId99" ref="A51"/>
-    <hyperlink r:id="rId100" ref="C51"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="A3" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="C3" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="A4" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="C4" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="A5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="C5" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="A6" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="C6" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="A7" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="C7" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="A8" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="C8" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="A9" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="C9" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="A10" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="C10" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="A11" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="C11" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="A12" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="C12" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="A13" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="C13" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="A14" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="C14" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="A15" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="C15" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="A16" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="C16" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="A17" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="C17" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="A18" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="C18" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="A19" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="C19" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="A20" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="C20" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="A21" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="C21" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="A22" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="C22" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="A23" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="C23" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="A24" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="C24" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="A25" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="C25" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="A26" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="C26" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="A27" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="C27" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="A28" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="C28" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="A29" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="C29" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="A30" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="C30" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="A31" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="C31" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="A32" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="C32" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="A33" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="C33" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="A34" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="C34" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="A35" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="C35" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="A36" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="C36" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="A37" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="C37" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="A38" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="C38" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="A39" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="C39" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="A40" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="C40" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="A41" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="C41" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="A42" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="C42" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="A43" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="C43" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="A44" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="C44" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="A45" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="C45" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="A46" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="C46" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="A47" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="C47" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="A48" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="C48" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="A49" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="C49" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="A50" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="C50" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="A51" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="C51" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
   </hyperlinks>
-  <drawing r:id="rId101"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId103"/>
+    <tablePart r:id="rId101"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>